<commit_message>
TMTI0045472 feb 26 24 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeRecordManagerForFVASupervisorUserOntheSFLightningView.xlsx
+++ b/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeRecordManagerForFVASupervisorUserOntheSFLightningView.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6FAEF65-0EA4-49B9-A375-B5AAFF807943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF3EE0F-A332-473E-8C17-26E1C276C3F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
   <si>
     <t>Global Search User</t>
   </si>
@@ -160,6 +160,36 @@
   </si>
   <si>
     <t>Abrams Capital – Loar Group - 27228</t>
+  </si>
+  <si>
+    <t>Eric Blackman</t>
+  </si>
+  <si>
+    <t>Time Tracking Beta Supervisor</t>
+  </si>
+  <si>
+    <t>Aamir Mansuri</t>
+  </si>
+  <si>
+    <t>Assistant Manager</t>
+  </si>
+  <si>
+    <t>Project Brown-STS Metals, Inc.-FVA-118279</t>
+  </si>
+  <si>
+    <t>Project Brown - FVA - 118279</t>
+  </si>
+  <si>
+    <t>Ashley Choi</t>
+  </si>
+  <si>
+    <t>Closing/Bring Down</t>
+  </si>
+  <si>
+    <t>Fieldwork</t>
+  </si>
+  <si>
+    <t>DetailLogsTIme</t>
   </si>
 </sst>
 </file>
@@ -496,15 +526,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -515,7 +546,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -526,14 +557,28 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
       <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
         <v>27</v>
       </c>
     </row>
@@ -588,7 +633,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
@@ -650,6 +695,17 @@
         <v>3</v>
       </c>
     </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -658,7 +714,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" bestFit="1" customWidth="1"/>
@@ -720,6 +776,17 @@
         <v>3</v>
       </c>
     </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -728,7 +795,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.140625" bestFit="1" customWidth="1"/>
@@ -757,6 +824,14 @@
         <v>38</v>
       </c>
       <c r="B3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s">
         <v>31</v>
       </c>
     </row>
@@ -810,7 +885,15 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="3"/>
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -820,7 +903,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C72E838B-CDBC-4DB0-BF1D-AC44E1CE047A}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
@@ -830,7 +913,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -850,6 +933,14 @@
       </c>
       <c r="B3" s="3" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>